<commit_message>
Synthèse : colonne « Montant envoyé à la logistique » par campagne
L'enveloppe totale envoyée (ex. 3 000 €) se saisit dans la Synthèse et
est comparée automatiquement aux factures justifiées de la campagne
(reste à justifier, % justifié). Campagnes adaptées au calendrier réel :
Rentrée scolaire, Noël, Pâques + opérations ponctuelles.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018pxe1k876zoUh9KcphmN1E
</commit_message>
<xml_diff>
--- a/gestion-dons-les-petits-enfants-de-marie.xlsx
+++ b/gestion-dons-les-petits-enfants-de-marie.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="96">
   <si>
     <t xml:space="preserve">GESTION DES DONS — LES PETITS ENFANTS DE MARIE</t>
   </si>
@@ -43,7 +43,7 @@
     <t xml:space="preserve">Synthèse</t>
   </si>
   <si>
-    <t xml:space="preserve">L'analyse comparative automatique par campagne de dons : entrées, dépenses, logistique, solde — et la clôture de l'année en bas du tableau. Rien à saisir ici.</t>
+    <t xml:space="preserve">L'analyse comparative par campagne : saisissez le montant total envoyé à la logistique (colonne jaune), le tableau le compare aux dons reçus et aux factures justifiées, et calcule le reste à justifier — avec la clôture de l'année en bas.</t>
   </si>
   <si>
     <t xml:space="preserve">Budget</t>
@@ -145,7 +145,7 @@
     <t xml:space="preserve">SYNTHÈSE PAR CAMPAGNE — ANALYSE COMPARATIVE</t>
   </si>
   <si>
-    <t xml:space="preserve">Tout se calcule automatiquement depuis l'onglet Trésorerie. Comparez les campagnes entre elles ; la dernière ligne donne la clôture de l'année.</t>
+    <t xml:space="preserve">Saisissez uniquement le « Montant envoyé à la logistique » (colonne jaune) : c'est l'enveloppe totale envoyée pour la campagne. Le reste se calcule depuis l'onglet Trésorerie (dons reçus, factures justifiées). La dernière ligne donne la clôture de l'année.</t>
   </si>
   <si>
     <t xml:space="preserve">Année :</t>
@@ -154,19 +154,19 @@
     <t xml:space="preserve">Dons reçus (€)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dépenses (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dont Logistique (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dont Achats articles (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solde (€)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% du don dépensé</t>
+    <t xml:space="preserve">Montant envoyé à la logistique (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factures justifiées (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reste à justifier (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solde campagne (€)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% de l'envoi justifié</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL — CLÔTURE DE L'ANNÉE</t>
@@ -304,7 +304,13 @@
     <t xml:space="preserve">Catégories de dépenses</t>
   </si>
   <si>
-    <t xml:space="preserve">Sans-abri France 2026</t>
+    <t xml:space="preserve">Rentrée scolaire 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rentrée scolaire 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opérations ponctuelles 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Autre</t>
@@ -1147,7 +1153,7 @@
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="n">
         <f aca="false">SUM(F7:F306)</f>
-        <v>500</v>
+        <v>3200</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="13" t="n">
@@ -1157,7 +1163,7 @@
       <c r="D5" s="13"/>
       <c r="E5" s="14" t="n">
         <f aca="false">SUM(F7:F306)-SUM(G7:G306)</f>
-        <v>160</v>
+        <v>2860</v>
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="15" t="n">
@@ -1207,12 +1213,12 @@
       </c>
       <c r="E7" s="19"/>
       <c r="F7" s="20" t="n">
-        <v>500</v>
+        <v>3200</v>
       </c>
       <c r="G7" s="20"/>
       <c r="H7" s="21" t="n">
         <f aca="false">IF(AND(F7="",G7=""),"",SUM(F$7:F7)-SUM(G$7:G7))</f>
-        <v>500</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1237,7 +1243,7 @@
       </c>
       <c r="H8" s="21" t="n">
         <f aca="false">IF(AND(F8="",G8=""),"",SUM(F$7:F8)-SUM(G$7:G8))</f>
-        <v>240</v>
+        <v>2940</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1262,7 +1268,7 @@
       </c>
       <c r="H9" s="21" t="n">
         <f aca="false">IF(AND(F9="",G9=""),"",SUM(F$7:F9)-SUM(G$7:G9))</f>
-        <v>160</v>
+        <v>2860</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5175,12 +5181,13 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5239,180 +5246,164 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="str">
         <f aca="false">IF(Listes!A5="","",Listes!A5)</f>
-        <v>Noël 2025</v>
+        <v>Rentrée scolaire 2025</v>
       </c>
       <c r="B6" s="25" t="n">
         <f aca="false">IF($A6="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A6))</f>
-        <v>500</v>
-      </c>
-      <c r="C6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="20"/>
+      <c r="D6" s="25" t="n">
         <f aca="false">IF($A6="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A6))</f>
-        <v>340</v>
-      </c>
-      <c r="D6" s="25" t="n">
-        <f aca="false">IF($A6="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A6,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v>80</v>
-      </c>
-      <c r="E6" s="25" t="n">
-        <f aca="false">IF($A6="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A6,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
-        <v>260</v>
+        <v>0</v>
+      </c>
+      <c r="E6" s="25" t="str">
+        <f aca="false">IF(OR($A6="",C6=""),"",C6-D6)</f>
+        <v/>
       </c>
       <c r="F6" s="21" t="n">
-        <f aca="false">IF($A6="","",B6-C6)</f>
-        <v>160</v>
-      </c>
-      <c r="G6" s="26" t="n">
-        <f aca="false">IF(OR($A6="",B6=0),"",C6/B6)</f>
-        <v>0.68</v>
+        <f aca="false">IF($A6="","",B6-IF(C6="",0,C6))</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="26" t="str">
+        <f aca="false">IF(OR($A6="",C6="",C6=0),"",D6/C6)</f>
+        <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="str">
         <f aca="false">IF(Listes!A6="","",Listes!A6)</f>
-        <v>Pâques 2026</v>
+        <v>Noël 2025</v>
       </c>
       <c r="B7" s="25" t="n">
         <f aca="false">IF($A7="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A7))</f>
-        <v>0</v>
-      </c>
-      <c r="C7" s="25" t="n">
+        <v>3200</v>
+      </c>
+      <c r="C7" s="20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D7" s="25" t="n">
         <f aca="false">IF($A7="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A7))</f>
-        <v>0</v>
-      </c>
-      <c r="D7" s="25" t="n">
-        <f aca="false">IF($A7="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A7,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v>0</v>
+        <v>340</v>
       </c>
       <c r="E7" s="25" t="n">
-        <f aca="false">IF($A7="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A7,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
-        <v>0</v>
+        <f aca="false">IF(OR($A7="",C7=""),"",C7-D7)</f>
+        <v>2660</v>
       </c>
       <c r="F7" s="21" t="n">
-        <f aca="false">IF($A7="","",B7-C7)</f>
-        <v>0</v>
-      </c>
-      <c r="G7" s="26" t="str">
-        <f aca="false">IF(OR($A7="",B7=0),"",C7/B7)</f>
-        <v/>
+        <f aca="false">IF($A7="","",B7-IF(C7="",0,C7))</f>
+        <v>200</v>
+      </c>
+      <c r="G7" s="26" t="n">
+        <f aca="false">IF(OR($A7="",C7="",C7=0),"",D7/C7)</f>
+        <v>0.113333333333333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="str">
         <f aca="false">IF(Listes!A7="","",Listes!A7)</f>
-        <v>Rentrée 2026</v>
+        <v>Pâques 2026</v>
       </c>
       <c r="B8" s="25" t="n">
         <f aca="false">IF($A8="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A8))</f>
         <v>0</v>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="C8" s="20"/>
+      <c r="D8" s="25" t="n">
         <f aca="false">IF($A8="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A8))</f>
         <v>0</v>
       </c>
-      <c r="D8" s="25" t="n">
-        <f aca="false">IF($A8="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A8,Trésorerie!$C$7:$C$306,"Logistique"))</f>
+      <c r="E8" s="25" t="str">
+        <f aca="false">IF(OR($A8="",C8=""),"",C8-D8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="21" t="n">
+        <f aca="false">IF($A8="","",B8-IF(C8="",0,C8))</f>
         <v>0</v>
       </c>
-      <c r="E8" s="25" t="n">
-        <f aca="false">IF($A8="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A8,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="21" t="n">
-        <f aca="false">IF($A8="","",B8-C8)</f>
-        <v>0</v>
-      </c>
       <c r="G8" s="26" t="str">
-        <f aca="false">IF(OR($A8="",B8=0),"",C8/B8)</f>
+        <f aca="false">IF(OR($A8="",C8="",C8=0),"",D8/C8)</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="24" t="str">
         <f aca="false">IF(Listes!A8="","",Listes!A8)</f>
-        <v>Noël 2026</v>
+        <v>Rentrée scolaire 2026</v>
       </c>
       <c r="B9" s="25" t="n">
         <f aca="false">IF($A9="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A9))</f>
         <v>0</v>
       </c>
-      <c r="C9" s="25" t="n">
+      <c r="C9" s="20"/>
+      <c r="D9" s="25" t="n">
         <f aca="false">IF($A9="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A9))</f>
         <v>0</v>
       </c>
-      <c r="D9" s="25" t="n">
-        <f aca="false">IF($A9="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A9,Trésorerie!$C$7:$C$306,"Logistique"))</f>
+      <c r="E9" s="25" t="str">
+        <f aca="false">IF(OR($A9="",C9=""),"",C9-D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="21" t="n">
+        <f aca="false">IF($A9="","",B9-IF(C9="",0,C9))</f>
         <v>0</v>
       </c>
-      <c r="E9" s="25" t="n">
-        <f aca="false">IF($A9="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A9,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="21" t="n">
-        <f aca="false">IF($A9="","",B9-C9)</f>
-        <v>0</v>
-      </c>
       <c r="G9" s="26" t="str">
-        <f aca="false">IF(OR($A9="",B9=0),"",C9/B9)</f>
+        <f aca="false">IF(OR($A9="",C9="",C9=0),"",D9/C9)</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="24" t="str">
         <f aca="false">IF(Listes!A9="","",Listes!A9)</f>
-        <v>Sans-abri France 2026</v>
+        <v>Noël 2026</v>
       </c>
       <c r="B10" s="25" t="n">
         <f aca="false">IF($A10="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A10))</f>
         <v>0</v>
       </c>
-      <c r="C10" s="25" t="n">
+      <c r="C10" s="20"/>
+      <c r="D10" s="25" t="n">
         <f aca="false">IF($A10="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A10))</f>
         <v>0</v>
       </c>
-      <c r="D10" s="25" t="n">
-        <f aca="false">IF($A10="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A10,Trésorerie!$C$7:$C$306,"Logistique"))</f>
+      <c r="E10" s="25" t="str">
+        <f aca="false">IF(OR($A10="",C10=""),"",C10-D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="21" t="n">
+        <f aca="false">IF($A10="","",B10-IF(C10="",0,C10))</f>
         <v>0</v>
       </c>
-      <c r="E10" s="25" t="n">
-        <f aca="false">IF($A10="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A10,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="21" t="n">
-        <f aca="false">IF($A10="","",B10-C10)</f>
-        <v>0</v>
-      </c>
       <c r="G10" s="26" t="str">
-        <f aca="false">IF(OR($A10="",B10=0),"",C10/B10)</f>
+        <f aca="false">IF(OR($A10="",C10="",C10=0),"",D10/C10)</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="str">
         <f aca="false">IF(Listes!A10="","",Listes!A10)</f>
-        <v/>
-      </c>
-      <c r="B11" s="25" t="str">
+        <v>Opérations ponctuelles 2026</v>
+      </c>
+      <c r="B11" s="25" t="n">
         <f aca="false">IF($A11="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A11))</f>
-        <v/>
-      </c>
-      <c r="C11" s="25" t="str">
+        <v>0</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="25" t="n">
         <f aca="false">IF($A11="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A11))</f>
-        <v/>
-      </c>
-      <c r="D11" s="25" t="str">
-        <f aca="false">IF($A11="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A11,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="E11" s="25" t="str">
-        <f aca="false">IF($A11="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A11,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
-        <v/>
-      </c>
-      <c r="F11" s="21" t="str">
-        <f aca="false">IF($A11="","",B11-C11)</f>
-        <v/>
+        <f aca="false">IF(OR($A11="",C11=""),"",C11-D11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="21" t="n">
+        <f aca="false">IF($A11="","",B11-IF(C11="",0,C11))</f>
+        <v>0</v>
       </c>
       <c r="G11" s="26" t="str">
-        <f aca="false">IF(OR($A11="",B11=0),"",C11/B11)</f>
+        <f aca="false">IF(OR($A11="",C11="",C11=0),"",D11/C11)</f>
         <v/>
       </c>
     </row>
@@ -5425,24 +5416,21 @@
         <f aca="false">IF($A12="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A12))</f>
         <v/>
       </c>
-      <c r="C12" s="25" t="str">
+      <c r="C12" s="20"/>
+      <c r="D12" s="25" t="str">
         <f aca="false">IF($A12="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A12))</f>
         <v/>
       </c>
-      <c r="D12" s="25" t="str">
-        <f aca="false">IF($A12="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A12,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v/>
-      </c>
       <c r="E12" s="25" t="str">
-        <f aca="false">IF($A12="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A12,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
+        <f aca="false">IF(OR($A12="",C12=""),"",C12-D12)</f>
         <v/>
       </c>
       <c r="F12" s="21" t="str">
-        <f aca="false">IF($A12="","",B12-C12)</f>
+        <f aca="false">IF($A12="","",B12-IF(C12="",0,C12))</f>
         <v/>
       </c>
       <c r="G12" s="26" t="str">
-        <f aca="false">IF(OR($A12="",B12=0),"",C12/B12)</f>
+        <f aca="false">IF(OR($A12="",C12="",C12=0),"",D12/C12)</f>
         <v/>
       </c>
     </row>
@@ -5455,24 +5443,21 @@
         <f aca="false">IF($A13="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A13))</f>
         <v/>
       </c>
-      <c r="C13" s="25" t="str">
+      <c r="C13" s="20"/>
+      <c r="D13" s="25" t="str">
         <f aca="false">IF($A13="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A13))</f>
         <v/>
       </c>
-      <c r="D13" s="25" t="str">
-        <f aca="false">IF($A13="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A13,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v/>
-      </c>
       <c r="E13" s="25" t="str">
-        <f aca="false">IF($A13="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A13,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
+        <f aca="false">IF(OR($A13="",C13=""),"",C13-D13)</f>
         <v/>
       </c>
       <c r="F13" s="21" t="str">
-        <f aca="false">IF($A13="","",B13-C13)</f>
+        <f aca="false">IF($A13="","",B13-IF(C13="",0,C13))</f>
         <v/>
       </c>
       <c r="G13" s="26" t="str">
-        <f aca="false">IF(OR($A13="",B13=0),"",C13/B13)</f>
+        <f aca="false">IF(OR($A13="",C13="",C13=0),"",D13/C13)</f>
         <v/>
       </c>
     </row>
@@ -5485,24 +5470,21 @@
         <f aca="false">IF($A14="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A14))</f>
         <v/>
       </c>
-      <c r="C14" s="25" t="str">
+      <c r="C14" s="20"/>
+      <c r="D14" s="25" t="str">
         <f aca="false">IF($A14="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A14))</f>
         <v/>
       </c>
-      <c r="D14" s="25" t="str">
-        <f aca="false">IF($A14="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A14,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v/>
-      </c>
       <c r="E14" s="25" t="str">
-        <f aca="false">IF($A14="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A14,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
+        <f aca="false">IF(OR($A14="",C14=""),"",C14-D14)</f>
         <v/>
       </c>
       <c r="F14" s="21" t="str">
-        <f aca="false">IF($A14="","",B14-C14)</f>
+        <f aca="false">IF($A14="","",B14-IF(C14="",0,C14))</f>
         <v/>
       </c>
       <c r="G14" s="26" t="str">
-        <f aca="false">IF(OR($A14="",B14=0),"",C14/B14)</f>
+        <f aca="false">IF(OR($A14="",C14="",C14=0),"",D14/C14)</f>
         <v/>
       </c>
     </row>
@@ -5515,24 +5497,21 @@
         <f aca="false">IF($A15="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A15))</f>
         <v/>
       </c>
-      <c r="C15" s="25" t="str">
+      <c r="C15" s="20"/>
+      <c r="D15" s="25" t="str">
         <f aca="false">IF($A15="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A15))</f>
         <v/>
       </c>
-      <c r="D15" s="25" t="str">
-        <f aca="false">IF($A15="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A15,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v/>
-      </c>
       <c r="E15" s="25" t="str">
-        <f aca="false">IF($A15="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A15,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
+        <f aca="false">IF(OR($A15="",C15=""),"",C15-D15)</f>
         <v/>
       </c>
       <c r="F15" s="21" t="str">
-        <f aca="false">IF($A15="","",B15-C15)</f>
+        <f aca="false">IF($A15="","",B15-IF(C15="",0,C15))</f>
         <v/>
       </c>
       <c r="G15" s="26" t="str">
-        <f aca="false">IF(OR($A15="",B15=0),"",C15/B15)</f>
+        <f aca="false">IF(OR($A15="",C15="",C15=0),"",D15/C15)</f>
         <v/>
       </c>
     </row>
@@ -5545,24 +5524,21 @@
         <f aca="false">IF($A16="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A16))</f>
         <v/>
       </c>
-      <c r="C16" s="25" t="str">
+      <c r="C16" s="20"/>
+      <c r="D16" s="25" t="str">
         <f aca="false">IF($A16="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A16))</f>
         <v/>
       </c>
-      <c r="D16" s="25" t="str">
-        <f aca="false">IF($A16="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A16,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v/>
-      </c>
       <c r="E16" s="25" t="str">
-        <f aca="false">IF($A16="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A16,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
+        <f aca="false">IF(OR($A16="",C16=""),"",C16-D16)</f>
         <v/>
       </c>
       <c r="F16" s="21" t="str">
-        <f aca="false">IF($A16="","",B16-C16)</f>
+        <f aca="false">IF($A16="","",B16-IF(C16="",0,C16))</f>
         <v/>
       </c>
       <c r="G16" s="26" t="str">
-        <f aca="false">IF(OR($A16="",B16=0),"",C16/B16)</f>
+        <f aca="false">IF(OR($A16="",C16="",C16=0),"",D16/C16)</f>
         <v/>
       </c>
     </row>
@@ -5575,24 +5551,21 @@
         <f aca="false">IF($A17="","",SUMIFS(Trésorerie!$F$7:$F$306,Trésorerie!$B$7:$B$306,$A17))</f>
         <v/>
       </c>
-      <c r="C17" s="25" t="str">
+      <c r="C17" s="20"/>
+      <c r="D17" s="25" t="str">
         <f aca="false">IF($A17="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A17))</f>
         <v/>
       </c>
-      <c r="D17" s="25" t="str">
-        <f aca="false">IF($A17="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A17,Trésorerie!$C$7:$C$306,"Logistique"))</f>
-        <v/>
-      </c>
       <c r="E17" s="25" t="str">
-        <f aca="false">IF($A17="","",SUMIFS(Trésorerie!$G$7:$G$306,Trésorerie!$B$7:$B$306,$A17,Trésorerie!$C$7:$C$306,"Achats articles"))</f>
+        <f aca="false">IF(OR($A17="",C17=""),"",C17-D17)</f>
         <v/>
       </c>
       <c r="F17" s="21" t="str">
-        <f aca="false">IF($A17="","",B17-C17)</f>
+        <f aca="false">IF($A17="","",B17-IF(C17="",0,C17))</f>
         <v/>
       </c>
       <c r="G17" s="26" t="str">
-        <f aca="false">IF(OR($A17="",B17=0),"",C17/B17)</f>
+        <f aca="false">IF(OR($A17="",C17="",C17=0),"",D17/C17)</f>
         <v/>
       </c>
     </row>
@@ -5602,27 +5575,27 @@
       </c>
       <c r="B18" s="28" t="n">
         <f aca="false">SUM(B6:B17)</f>
-        <v>500</v>
+        <v>3200</v>
       </c>
       <c r="C18" s="28" t="n">
         <f aca="false">SUM(C6:C17)</f>
-        <v>340</v>
+        <v>3000</v>
       </c>
       <c r="D18" s="28" t="n">
         <f aca="false">SUM(D6:D17)</f>
-        <v>80</v>
+        <v>340</v>
       </c>
       <c r="E18" s="28" t="n">
         <f aca="false">SUM(E6:E17)</f>
-        <v>260</v>
+        <v>2660</v>
       </c>
       <c r="F18" s="28" t="n">
         <f aca="false">SUM(F6:F17)</f>
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="G18" s="29" t="n">
-        <f aca="false">IF(B18=0,"",C18/B18)</f>
-        <v>0.68</v>
+        <f aca="false">IF(C18=0,"",D18/C18)</f>
+        <v>0.113333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -5639,7 +5612,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7562DE11-1096-4A31-ADF9-A3D033822195}</x14:id>
+          <x14:id>{2DD6E22C-EBAF-4E7F-97F0-409CCAA96739}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5655,7 +5628,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7562DE11-1096-4A31-ADF9-A3D033822195}">
+          <x14:cfRule type="dataBar" id="{2DD6E22C-EBAF-4E7F-97F0-409CCAA96739}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5946,7 +5919,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A0318FF6-B971-4179-8D52-4DFC417971D6}</x14:id>
+          <x14:id>{1D872821-6712-496D-B7E3-B4D28C6DE030}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5962,7 +5935,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A0318FF6-B971-4179-8D52-4DFC417971D6}">
+          <x14:cfRule type="dataBar" id="{1D872821-6712-496D-B7E3-B4D28C6DE030}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -9145,7 +9118,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>30</v>
@@ -9153,7 +9126,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>32</v>
@@ -9161,7 +9134,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B7" s="18" t="s">
         <v>35</v>
@@ -9169,7 +9142,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="B8" s="18" t="s">
         <v>55</v>
@@ -9177,16 +9150,18 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18"/>
+      <c r="A10" s="18" t="s">
+        <v>94</v>
+      </c>
       <c r="B10" s="18" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>